<commit_message>
feature: excel 'empresa per mida y provincia' changed and graphics made
</commit_message>
<xml_diff>
--- a/data/Empresa per mida y provincia 2008-2022.xlsx
+++ b/data/Empresa per mida y provincia 2008-2022.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\miria\OneDrive - Universitat Politècnica de Catalunya\Personal\HACKATON\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{840B89C9-7736-4258-B5FE-BAB9836F4ABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14166926-9E4C-4173-9532-55A365A7965F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4EEA3490-7564-45D2-A2CA-A64496852BF8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="98">
   <si>
     <t>CCAA</t>
   </si>
@@ -365,11 +365,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -869,13 +868,13 @@
       <c r="D1" t="s">
         <v>84</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" t="s">
         <v>70</v>
       </c>
       <c r="F1" t="s">
         <v>85</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" t="s">
         <v>71</v>
       </c>
       <c r="H1" s="2" t="s">
@@ -923,7 +922,7 @@
       <c r="V1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="W1" t="s">
         <v>79</v>
       </c>
       <c r="X1" s="2" t="s">
@@ -3988,6 +3987,9 @@
       </c>
     </row>
     <row r="35" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
+        <v>33</v>
+      </c>
       <c r="C35" t="s">
         <v>35</v>
       </c>
@@ -4077,6 +4079,9 @@
       </c>
     </row>
     <row r="36" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B36" t="s">
+        <v>33</v>
+      </c>
       <c r="C36" t="s">
         <v>36</v>
       </c>
@@ -4166,6 +4171,9 @@
       </c>
     </row>
     <row r="37" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B37" t="s">
+        <v>33</v>
+      </c>
       <c r="C37" t="s">
         <v>37</v>
       </c>
@@ -4255,6 +4263,9 @@
       </c>
     </row>
     <row r="38" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B38" t="s">
+        <v>33</v>
+      </c>
       <c r="C38" t="s">
         <v>38</v>
       </c>
@@ -4344,6 +4355,9 @@
       </c>
     </row>
     <row r="39" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B39" t="s">
+        <v>33</v>
+      </c>
       <c r="C39" t="s">
         <v>2</v>
       </c>
@@ -4525,6 +4539,9 @@
       </c>
     </row>
     <row r="41" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B41" t="s">
+        <v>39</v>
+      </c>
       <c r="C41" t="s">
         <v>41</v>
       </c>
@@ -4614,6 +4631,9 @@
       </c>
     </row>
     <row r="42" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B42" t="s">
+        <v>39</v>
+      </c>
       <c r="C42" t="s">
         <v>42</v>
       </c>
@@ -4703,6 +4723,9 @@
       </c>
     </row>
     <row r="43" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B43" t="s">
+        <v>39</v>
+      </c>
       <c r="C43" t="s">
         <v>43</v>
       </c>
@@ -4792,6 +4815,9 @@
       </c>
     </row>
     <row r="44" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B44" t="s">
+        <v>39</v>
+      </c>
       <c r="C44" t="s">
         <v>2</v>
       </c>
@@ -4973,6 +4999,9 @@
       </c>
     </row>
     <row r="46" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B46" t="s">
+        <v>44</v>
+      </c>
       <c r="C46" t="s">
         <v>2</v>
       </c>
@@ -5154,6 +5183,9 @@
       </c>
     </row>
     <row r="48" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B48" t="s">
+        <v>45</v>
+      </c>
       <c r="C48" t="s">
         <v>47</v>
       </c>
@@ -5243,6 +5275,9 @@
       </c>
     </row>
     <row r="49" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B49" t="s">
+        <v>45</v>
+      </c>
       <c r="C49" t="s">
         <v>48</v>
       </c>
@@ -5332,6 +5367,9 @@
       </c>
     </row>
     <row r="50" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B50" t="s">
+        <v>45</v>
+      </c>
       <c r="C50" t="s">
         <v>2</v>
       </c>
@@ -5513,6 +5551,9 @@
       </c>
     </row>
     <row r="52" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B52" t="s">
+        <v>49</v>
+      </c>
       <c r="C52" t="s">
         <v>51</v>
       </c>
@@ -5602,6 +5643,9 @@
       </c>
     </row>
     <row r="53" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B53" t="s">
+        <v>49</v>
+      </c>
       <c r="C53" t="s">
         <v>2</v>
       </c>
@@ -5783,6 +5827,9 @@
       </c>
     </row>
     <row r="55" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B55" t="s">
+        <v>52</v>
+      </c>
       <c r="C55" t="s">
         <v>54</v>
       </c>
@@ -5872,6 +5919,9 @@
       </c>
     </row>
     <row r="56" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B56" t="s">
+        <v>52</v>
+      </c>
       <c r="C56" t="s">
         <v>55</v>
       </c>
@@ -5961,6 +6011,9 @@
       </c>
     </row>
     <row r="57" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B57" t="s">
+        <v>52</v>
+      </c>
       <c r="C57" t="s">
         <v>56</v>
       </c>
@@ -6050,6 +6103,9 @@
       </c>
     </row>
     <row r="58" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B58" t="s">
+        <v>52</v>
+      </c>
       <c r="C58" t="s">
         <v>2</v>
       </c>
@@ -6231,6 +6287,9 @@
       </c>
     </row>
     <row r="60" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B60" t="s">
+        <v>57</v>
+      </c>
       <c r="C60" t="s">
         <v>2</v>
       </c>
@@ -6412,6 +6471,9 @@
       </c>
     </row>
     <row r="62" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B62" t="s">
+        <v>59</v>
+      </c>
       <c r="C62" t="s">
         <v>2</v>
       </c>
@@ -6593,6 +6655,9 @@
       </c>
     </row>
     <row r="64" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B64" t="s">
+        <v>60</v>
+      </c>
       <c r="C64" t="s">
         <v>2</v>
       </c>
@@ -6774,6 +6839,9 @@
       </c>
     </row>
     <row r="66" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B66" t="s">
+        <v>62</v>
+      </c>
       <c r="C66" t="s">
         <v>2</v>
       </c>
@@ -6955,6 +7023,9 @@
       </c>
     </row>
     <row r="68" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B68" t="s">
+        <v>64</v>
+      </c>
       <c r="C68" t="s">
         <v>66</v>
       </c>
@@ -7044,6 +7115,9 @@
       </c>
     </row>
     <row r="69" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B69" t="s">
+        <v>64</v>
+      </c>
       <c r="C69" t="s">
         <v>67</v>
       </c>
@@ -7133,6 +7207,9 @@
       </c>
     </row>
     <row r="70" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B70" t="s">
+        <v>64</v>
+      </c>
       <c r="C70" t="s">
         <v>2</v>
       </c>
@@ -7314,6 +7391,9 @@
       </c>
     </row>
     <row r="72" spans="2:31" x14ac:dyDescent="0.3">
+      <c r="B72" t="s">
+        <v>68</v>
+      </c>
       <c r="C72" t="s">
         <v>2</v>
       </c>

</xml_diff>